<commit_message>
feat(comms): pristine Office templates with Brand Kit logo injection
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/templates/office/xlsx/formal-grievance_blue.xlsx
+++ b/public/templates/office/xlsx/formal-grievance_blue.xlsx
@@ -4,47 +4,53 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Details" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Steps" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="11">
   <si>
     <t>Local</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>Title</t>
   </si>
   <si>
+    <t>Member</t>
+  </si>
+  <si>
     <t>Date</t>
   </si>
   <si>
-    <t>Time</t>
-  </si>
-  <si>
-    <t>Location</t>
-  </si>
-  <si>
-    <t>Member</t>
-  </si>
-  <si>
-    <t>Steward / Contact</t>
-  </si>
-  <si>
-    <t>Body</t>
-  </si>
-  <si>
-    <t>CTA / Headline</t>
+    <t>Step</t>
+  </si>
+  <si>
+    <t>Action</t>
+  </si>
+  <si>
+    <t>Owner</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Open</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -56,8 +62,11 @@
       <b/>
       <color rgb="FFFFFFFF"/>
     </font>
+    <font>
+      <b/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -67,6 +76,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1B4F72"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8EEF4"/>
       </patternFill>
     </fill>
   </fills>
@@ -82,9 +96,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -424,57 +439,72 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="48" customWidth="1"/>
-    <col min="3" max="3" width="28" customWidth="1"/>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="36" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>8</v>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>1</v>
+      </c>
+      <c r="E6" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>